<commit_message>
RE-041.4: Dry Powder Ledger adapter, joins live episode + manual ledger
</commit_message>
<xml_diff>
--- a/data/raw/dry_powder_ledger.xlsx
+++ b/data/raw/dry_powder_ledger.xlsx
@@ -650,7 +650,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Fecha (AAAA.MM.DD o AAAA.MM)</t>
+          <t>Fecha (calendario real, AAAA-MM-DD)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -850,7 +850,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Fecha (AAAA.MM.DD o AAAA.MM)</t>
+          <t>Fecha (calendario real, AAAA-MM-DD)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">

</xml_diff>

<commit_message>
RE-041.6: add Activo/Instrumento column to Dry Powder Ledger
</commit_message>
<xml_diff>
--- a/data/raw/dry_powder_ledger.xlsx
+++ b/data/raw/dry_powder_ledger.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17260" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,14 +11,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AML" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,8 +28,21 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -69,16 +81,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -442,93 +467,114 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="109.5" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>DRY POWDER LEDGER — Notas de uso</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="3" ht="64" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Propósito</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Registro manual operado por Armando para las cinco entradas de DryPowderProtocolInputs (engine/dry_powder_protocol.py) que ningún dato de mercado puede observar: pólvora seca inicial del episodio, capital acumulado desplegado, postura más alta alcanzada, y los dos campos de cadencia (días/pp desde el último tramo). No sustituye al protocolo -- alimenta al futuro adaptador que construya DryPowderProtocolInputs a partir de este archivo cruzado con engine/live_episode.py.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="7" t="n"/>
+      <c r="B4" s="5" t="n"/>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Separado de personal_capacity_facts.xlsx</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>personal_capacity_facts.xlsx es una foto estática (9 hechos, se reescribe). Este archivo es un registro que crece con cada tramo ejecutado -- misma separación de responsabilidad que ya existe entre shiller.xlsx (mercado) y personal_capacity_facts.xlsx (capacidad).</t>
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="7" t="n"/>
+      <c r="B6" s="5" t="n"/>
+    </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Código de color</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="B7" s="5" t="n"/>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Azul</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Valor manual -- lo escribe Armando.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="5" t="n"/>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Cuándo rellenar la Sección 1 (Episodio actual)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Solo cuando engine/live_episode.py detecte un episodio activo por primera vez. Mientras no haya episodio (caso de hoy, 2026-08-10: mercado en máximo histórico), esta sección queda en 'Pendiente' -- no es un dato que falte, es que la pregunta no aplica todavía.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="5" t="n"/>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Cuándo añadir una fila a la Sección 2 (Registro de tramos)</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Cada vez que se ejecuta realmente un tramo (dinero movido, no una decisión sobre el papel). Fecha, importe, y la postura combinada vigente en ese momento -- los demás campos (pp de caída acumulada, días desde el último tramo, capital acumulado) se derivan cruzando estas filas con los datos de Shiller, no se escriben a mano.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="5" t="n"/>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Qué pasa si empieza un episodio nuevo</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>El ratchet de RE-041.1 solo se reinicia con una recuperación completa a un nuevo máximo (misma definición de episodio que drawdown_engine.py). Cuando eso ocurra, actualizar la Sección 1 con la nueva fecha/pólvora seca -- las filas antiguas de la Sección 2 NO se borran, quedan como historial; el futuro adaptador filtra por fecha &gt;= inicio del episodio vigente.</t>
         </is>
@@ -545,16 +591,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>DRY POWDER LEDGER — AMS</t>
@@ -562,44 +609,44 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>1. EPISODIO ACTUAL (marcador, una fila por episodio activo)</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Fecha inicio episodio (formato Shiller AAAA.MM)</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -616,12 +663,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Pólvora seca inicial del episodio (€)</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -638,96 +685,111 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>2. REGISTRO DE TRAMOS DESPLEGADOS (una fila por compra ejecutada, nunca se borra)</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Fecha (calendario real, AAAA-MM-DD)</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Importe desplegado (€)</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Postura vigente</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Activo / Instrumento</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="10" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
+      <c r="A11" s="2" t="n"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="10" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="10" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n"/>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="10" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n"/>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n"/>
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="3" t="n"/>
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="10" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n"/>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="10" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -745,16 +807,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>DRY POWDER LEDGER — AML</t>
@@ -762,44 +825,44 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>1. EPISODIO ACTUAL (marcador, una fila por episodio activo)</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Fecha inicio episodio (formato Shiller AAAA.MM)</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -816,12 +879,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Pólvora seca inicial del episodio (€)</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -838,96 +901,111 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>2. REGISTRO DE TRAMOS DESPLEGADOS (una fila por compra ejecutada, nunca se borra)</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Fecha (calendario real, AAAA-MM-DD)</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Importe desplegado (€)</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Postura vigente</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Activo / Instrumento</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="10" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
+      <c r="A11" s="2" t="n"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="10" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="10" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n"/>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="10" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n"/>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n"/>
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="3" t="n"/>
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="10" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n"/>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="10" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Consolidación de cambios locales pendientes (datos + gate + docs)
</commit_message>
<xml_diff>
--- a/data/raw/dry_powder_ledger.xlsx
+++ b/data/raw/dry_powder_ledger.xlsx
@@ -1,18 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/armando/Library/Mobile Documents/com~apple~CloudDocs/12. FINANZAS/11. SOP/SOP_Research_Engine/data/raw/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_9A1750955E6C1357A1DF92F2481EDC22868B835C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Notas" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="AMS" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="AML" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Notas" sheetId="1" r:id="rId1"/>
+    <sheet name="AMS" sheetId="2" r:id="rId2"/>
+    <sheet name="AML" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -24,110 +29,107 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="32">
   <si>
-    <t xml:space="preserve">DRY POWDER LEDGER — Notas de uso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Propósito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Registro manual operado por Armando para las cinco entradas de DryPowderProtocolInputs (engine/dry_powder_protocol.py) que ningún dato de mercado puede observar: pólvora seca inicial del episodio, capital acumulado desplegado, postura más alta alcanzada, y los dos campos de cadencia (días/pp desde el último tramo). No sustituye al protocolo -- alimenta al futuro adaptador que construya DryPowderProtocolInputs a partir de este archivo cruzado con engine/live_episode.py.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Separado de personal_capacity_facts.xlsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">personal_capacity_facts.xlsx es una foto estática (9 hechos, se reescribe). Este archivo es un registro que crece con cada tramo ejecutado -- misma separación de responsabilidad que ya existe entre shiller.xlsx (mercado) y personal_capacity_facts.xlsx (capacidad).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Código de color</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Azul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor manual -- lo escribe Armando.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cuándo rellenar la Sección 1 (Episodio actual)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solo cuando engine/live_episode.py detecte un episodio activo por primera vez. Mientras no haya episodio (caso de hoy, 2026-08-10: mercado en máximo histórico), esta sección queda en 'Pendiente' -- no es un dato que falte, es que la pregunta no aplica todavía.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cuándo añadir una fila a la Sección 2 (Registro de tramos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cada vez que se ejecuta realmente un tramo (dinero movido, no una decisión sobre el papel). Fecha, importe, y la postura combinada vigente en ese momento -- los demás campos (pp de caída acumulada, días desde el último tramo, capital acumulado) se derivan cruzando estas filas con los datos de Shiller, no se escriben a mano.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Qué pasa si empieza un episodio nuevo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El ratchet de RE-041.1 solo se reinicia con una recuperación completa a un nuevo máximo (misma definición de episodio que drawdown_engine.py). Cuando eso ocurra, actualizar la Sección 1 con la nueva fecha/pólvora seca -- las filas antiguas de la Sección 2 NO se borran, quedan como historial; el futuro adaptador filtra por fecha &gt;= inicio del episodio vigente.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRY POWDER LEDGER — AMS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. EPISODIO ACTUAL (marcador, una fila por episodio activo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concepto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nota</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fecha inicio episodio (formato Shiller AAAA.MM)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pendiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rellenar solo cuando engine/live_episode.py confirme un episodio activo (detect_current_episode() no devuelve None). Debe coincidir con CurrentEpisode.peak_date de ese momento.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pólvora seca inicial del episodio (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Liquidez desplegable real el día de inicio del episodio, no hoy. Es la única cifra que nadie más que Armando puede conocer -- no se deriva de ningún dato de mercado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. REGISTRO DE TRAMOS DESPLEGADOS (una fila por compra ejecutada, nunca se borra)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fecha (calendario real, AAAA-MM-DD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Importe desplegado (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Postura vigente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Activo / Instrumento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRY POWDER LEDGER — AML</t>
+    <t>DRY POWDER LEDGER — Notas de uso</t>
+  </si>
+  <si>
+    <t>Propósito</t>
+  </si>
+  <si>
+    <t>Registro manual operado por Armando para las cinco entradas de DryPowderProtocolInputs (engine/dry_powder_protocol.py) que ningún dato de mercado puede observar: pólvora seca inicial del episodio, capital acumulado desplegado, postura más alta alcanzada, y los dos campos de cadencia (días/pp desde el último tramo). No sustituye al protocolo -- alimenta al futuro adaptador que construya DryPowderProtocolInputs a partir de este archivo cruzado con engine/live_episode.py.</t>
+  </si>
+  <si>
+    <t>Separado de personal_capacity_facts.xlsx</t>
+  </si>
+  <si>
+    <t>personal_capacity_facts.xlsx es una foto estática (9 hechos, se reescribe). Este archivo es un registro que crece con cada tramo ejecutado -- misma separación de responsabilidad que ya existe entre shiller.xlsx (mercado) y personal_capacity_facts.xlsx (capacidad).</t>
+  </si>
+  <si>
+    <t>Código de color</t>
+  </si>
+  <si>
+    <t>Azul</t>
+  </si>
+  <si>
+    <t>Valor manual -- lo escribe Armando.</t>
+  </si>
+  <si>
+    <t>Cuándo rellenar la Sección 1 (Episodio actual)</t>
+  </si>
+  <si>
+    <t>Solo cuando engine/live_episode.py detecte un episodio activo por primera vez. Mientras no haya episodio (caso de hoy, 2026-08-10: mercado en máximo histórico), esta sección queda en 'Pendiente' -- no es un dato que falte, es que la pregunta no aplica todavía.</t>
+  </si>
+  <si>
+    <t>Cuándo añadir una fila a la Sección 2 (Registro de tramos)</t>
+  </si>
+  <si>
+    <t>Cada vez que se ejecuta realmente un tramo (dinero movido, no una decisión sobre el papel). Fecha, importe, y la postura combinada vigente en ese momento -- los demás campos (pp de caída acumulada, días desde el último tramo, capital acumulado) se derivan cruzando estas filas con los datos de Shiller, no se escriben a mano.</t>
+  </si>
+  <si>
+    <t>Qué pasa si empieza un episodio nuevo</t>
+  </si>
+  <si>
+    <t>El ratchet de RE-041.1 solo se reinicia con una recuperación completa a un nuevo máximo (misma definición de episodio que drawdown_engine.py). Cuando eso ocurra, actualizar la Sección 1 con la nueva fecha/pólvora seca -- las filas antiguas de la Sección 2 NO se borran, quedan como historial; el futuro adaptador filtra por fecha &gt;= inicio del episodio vigente.</t>
+  </si>
+  <si>
+    <t>DRY POWDER LEDGER — AMS</t>
+  </si>
+  <si>
+    <t>1. EPISODIO ACTUAL (marcador, una fila por episodio activo)</t>
+  </si>
+  <si>
+    <t>Concepto</t>
+  </si>
+  <si>
+    <t>Valor</t>
+  </si>
+  <si>
+    <t>Fuente</t>
+  </si>
+  <si>
+    <t>Nota</t>
+  </si>
+  <si>
+    <t>Fecha inicio episodio (formato Shiller AAAA.MM)</t>
+  </si>
+  <si>
+    <t>Pendiente</t>
+  </si>
+  <si>
+    <t>Manual</t>
+  </si>
+  <si>
+    <t>Rellenar solo cuando engine/live_episode.py confirme un episodio activo (detect_current_episode() no devuelve None). Debe coincidir con CurrentEpisode.peak_date de ese momento.</t>
+  </si>
+  <si>
+    <t>Pólvora seca inicial del episodio (€)</t>
+  </si>
+  <si>
+    <t>Liquidez desplegable real el día de inicio del episodio, no hoy. Es la única cifra que nadie más que Armando puede conocer -- no se deriva de ningún dato de mercado.</t>
+  </si>
+  <si>
+    <t>2. REGISTRO DE TRAMOS DESPLEGADOS (una fila por compra ejecutada, nunca se borra)</t>
+  </si>
+  <si>
+    <t>Fecha (calendario real, AAAA-MM-DD)</t>
+  </si>
+  <si>
+    <t>Importe desplegado (€)</t>
+  </si>
+  <si>
+    <t>Postura vigente</t>
+  </si>
+  <si>
+    <t>Activo / Instrumento</t>
+  </si>
+  <si>
+    <t>DRY POWDER LEDGER — AML</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -136,29 +138,14 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="13"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -172,18 +159,16 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <name val="Cambria"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Cambria"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -207,7 +192,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -215,97 +200,50 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="14">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -364,13 +302,29 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -412,12 +366,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -446,7 +400,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -467,7 +421,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -518,7 +472,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -536,32 +490,31 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="109.5"/>
+    <col min="1" max="1" width="46" customWidth="1"/>
+    <col min="2" max="2" width="109.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:2" ht="63.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -569,11 +522,11 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="4"/>
       <c r="B4" s="3"/>
     </row>
-    <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -581,17 +534,17 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="4"/>
       <c r="B6" s="3"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="3"/>
     </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>6</v>
       </c>
@@ -599,11 +552,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="4"/>
       <c r="B9" s="3"/>
     </row>
-    <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -611,11 +564,11 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="4"/>
       <c r="B11" s="3"/>
     </row>
-    <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -623,11 +576,11 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="4"/>
       <c r="B13" s="3"/>
     </row>
-    <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -636,37 +589,29 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
+    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>15</v>
       </c>
@@ -674,7 +619,7 @@
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
         <v>16</v>
       </c>
@@ -688,7 +633,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:5" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>20</v>
       </c>
@@ -702,7 +647,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:5" ht="48" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>24</v>
       </c>
@@ -716,7 +661,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>26</v>
       </c>
@@ -724,7 +669,7 @@
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
         <v>27</v>
       </c>
@@ -741,70 +686,70 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="12"/>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
       <c r="E10" s="13"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="12"/>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
       <c r="E11" s="13"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="12"/>
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
       <c r="E12" s="13"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="12"/>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
       <c r="E13" s="13"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="12"/>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
       <c r="E14" s="13"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="12"/>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
       <c r="E15" s="13"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="12"/>
       <c r="B16" s="12"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
       <c r="E16" s="13"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="12"/>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
       <c r="E17" s="13"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="12"/>
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
       <c r="E18" s="13"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="12"/>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
@@ -813,42 +758,34 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C19" type="list">
+    <dataValidation type="list" allowBlank="1" sqref="C10:C19" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Conserve,Prepare,Deploy Partially,Deploy Aggressively,Blocked"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
+    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>15</v>
       </c>
@@ -856,7 +793,7 @@
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
         <v>16</v>
       </c>
@@ -870,7 +807,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:5" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>20</v>
       </c>
@@ -884,7 +821,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:5" ht="48" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>24</v>
       </c>
@@ -898,7 +835,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>26</v>
       </c>
@@ -906,7 +843,7 @@
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
         <v>27</v>
       </c>
@@ -923,70 +860,70 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="12"/>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
       <c r="E10" s="13"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="12"/>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
       <c r="E11" s="13"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="12"/>
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
       <c r="E12" s="13"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="12"/>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
       <c r="E13" s="13"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="12"/>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
       <c r="E14" s="13"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="12"/>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
       <c r="E15" s="13"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="12"/>
       <c r="B16" s="12"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
       <c r="E16" s="13"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="12"/>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
       <c r="E17" s="13"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="12"/>
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
       <c r="E18" s="13"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="12"/>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
@@ -995,17 +932,12 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C19" type="list">
+    <dataValidation type="list" allowBlank="1" sqref="C10:C19" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Conserve,Prepare,Deploy Partially,Deploy Aggressively,Blocked"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>